<commit_message>
feat(p0): T1.4 任务系统重做（target_id/target_count 分离）
- Quests 表新增 目标数量 列；QuestData 增加 target_count（默认 1）
- track_kill/track_collect 改用 target_count 判定，修复原来
  "击杀数 >= 敌人ID" 的语义混淆（敌人 ID 稍大就永远完不成）
- track_explore 坐标编码方式废弃，改为 track_explore_map：
  进入目标地图即完成（collect_count 复用到访计数）
- 收集任务改为"获得时"触发：新增 VM._gain_item 统一入口
  （购买/掉落走这里），修复原来"使用物品才算收集"的错误语义
- 移动成功后显式触发探索追踪，替换原来恒真条件的丑陋写法
- 任务日志渲染显示 x/y 进度；读档不再重复触发探索追踪
- 配置修正：赏金猎人任务指向敌人 6（原指向 5 变异鼠），
  收集任务目标改为猎枪(4)，探索任务目标改为地图 5（地下遗迹）
- 新增 tests/smoke_quest.py：三类任务判定/奖励/购买计入/存档往返
  全部断言通过
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -2348,7 +2348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2359,6 +2359,7 @@
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2389,15 +2390,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>目标数量</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>奖励经验</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>奖励金币</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>奖励物品</t>
         </is>
@@ -2426,12 +2432,15 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" t="n">
         <v>100</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>200</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -2457,15 +2466,18 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
         <v>200</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>500</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -2491,15 +2503,18 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
         <v>150</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>300</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -2525,15 +2540,18 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
         <v>300</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>800</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>9</t>
         </is>

</xml_diff>